<commit_message>
Nesta aula terminamos o exercicio app(tranformando dados em uma tabela excel e alimentado a mesma).
</commit_message>
<xml_diff>
--- a/aula12/Alunos.xlsx
+++ b/aula12/Alunos.xlsx
@@ -436,11 +436,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>Amanda</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C2" t="n">
         <v>1.7</v>

</xml_diff>

<commit_message>
Nesta aula iniciamos o exercicio, sobre o banco TABAJARA.
</commit_message>
<xml_diff>
--- a/aula12/Alunos.xlsx
+++ b/aula12/Alunos.xlsx
@@ -436,11 +436,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Amanda</t>
+          <t>Girassol</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="C2" t="n">
         <v>1.7</v>

</xml_diff>